<commit_message>
Mark Autocad 2027 as Latest version on both platforms
Source xlsx column B set to "Latest" for Autocad 2027 in Windows and
Macbook sheets; regenerated manifest. Selecting this software will
now apply the +₹500 (win) / +₹1500 (mac) latest-version surcharge.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Softwares.xlsx
+++ b/Softwares.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AshishKumar.Soni/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AshishKumar.Soni/quicksoftwares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ECEDD8A-0C5B-EA41-A03E-41F26166F25C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B063D9E-8CD3-A641-8731-EBF13F9C7924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" activeTab="1" xr2:uid="{348E5074-3515-0B4A-AB07-E04CD59ECA3F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="117">
   <si>
     <t>Software</t>
   </si>
@@ -384,7 +384,10 @@
     <t>Autocad 2027</t>
   </si>
   <si>
-    <t>Price</t>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Latest</t>
   </si>
 </sst>
 </file>
@@ -1347,8 +1350,8 @@
       <c r="A107" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B107" s="5">
-        <v>2000</v>
+      <c r="B107" s="5" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1773,8 +1776,8 @@
       <c r="A81" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B81" s="5">
-        <v>10000</v>
+      <c r="B81" s="5" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: add Link column to Softwares.xlsx and regenerate manifest
Added the Link column (C) to both Windows and Macbook sheets and
started filling in download URLs. Regenerated softwares-manifest.js
so the Download Now flow can offer real links.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Softwares.xlsx
+++ b/Softwares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AshishKumar.Soni/quicksoftwares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9EF3020-D6CB-AB40-935B-7D72B81EF629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B22D535E-8335-3941-B0EB-02267DFB9702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" xr2:uid="{348E5074-3515-0B4A-AB07-E04CD59ECA3F}"/>
+    <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="16920" activeTab="1" xr2:uid="{348E5074-3515-0B4A-AB07-E04CD59ECA3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Windows" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="119">
   <si>
     <t>Software</t>
   </si>
@@ -388,13 +388,19 @@
   </si>
   <si>
     <t>Latest</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>www.youtube.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -420,6 +426,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -460,10 +474,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -472,8 +487,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -806,92 +823,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A4B76ED-CF2B-0D46-BCA1-852CF354D9D5}">
-  <dimension ref="A1:B107"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.5" style="2" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="5"/>
+    <col min="3" max="3" width="63.83203125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -1358,6 +1382,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{B3BC29F9-7458-544D-BD0D-890D56F499F9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -1365,92 +1392,96 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BB426D-FBED-3542-BD04-64E6FFCD9253}">
-  <dimension ref="A1:B81"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.5" style="2" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="5"/>
+    <col min="3" max="3" width="51.1640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>

</xml_diff>